<commit_message>
datos: +0 Kino, +1 Pool hasta 2026-08-28
</commit_message>
<xml_diff>
--- a/data/loto_pool.xlsx
+++ b/data/loto_pool.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -793,6 +793,18 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28  Vie</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>08, 09, 18, 21, 28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>